<commit_message>
chore: catch-up commit for approved uncommitted work
</commit_message>
<xml_diff>
--- a/corpus_aggregate.xlsx
+++ b/corpus_aggregate.xlsx
@@ -12,6 +12,9 @@
     <sheet name="Top Dependencies" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Repos Per Pattern" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cross-Tabulation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Repos Per Domain" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Domain Failure Signatures" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Domain x Vertical" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -493,28 +496,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>539</v>
+        <v>1070</v>
       </c>
       <c r="C2" t="n">
-        <v>528</v>
+        <v>1032</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.0%</t>
+          <t>96.4%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>405</v>
+        <v>1302</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>4.5%</t>
         </is>
       </c>
     </row>
@@ -525,60 +528,60 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157</v>
+        <v>468</v>
       </c>
       <c r="C3" t="n">
-        <v>152</v>
+        <v>430</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>96.8%</t>
+          <t>91.9%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>519</v>
+        <v>998</v>
       </c>
       <c r="G3" t="n">
-        <v>50</v>
+        <v>215</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>21.5%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="C4" t="n">
-        <v>99</v>
+        <v>141</v>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>90.0%</t>
+          <t>99.3%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>423</v>
+        <v>268</v>
       </c>
       <c r="G4" t="n">
-        <v>185</v>
+        <v>7</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>43.7%</t>
+          <t>2.6%</t>
         </is>
       </c>
     </row>
@@ -589,188 +592,156 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="C5" t="n">
-        <v>39</v>
+        <v>102</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>79.6%</t>
+          <t>77.9%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>310</v>
+        <v>532</v>
       </c>
       <c r="G5" t="n">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>92</v>
       </c>
       <c r="C6" t="n">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>87.0%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>168</v>
+        <v>789</v>
       </c>
       <c r="G6" t="n">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="C7" t="n">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>125</v>
+        <v>328</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>92.9%</t>
+          <t>89.8%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>564</v>
+        <v>315</v>
       </c>
       <c r="G8" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>59.0%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G9" t="n">
         <v>7</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" t="n">
-        <v>7</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>70.0%</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>32</v>
-      </c>
-      <c r="G10" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>9.4%</t>
+          <t>5.3%</t>
         </is>
       </c>
     </row>
@@ -785,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -853,7 +824,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>510</v>
+        <v>961</v>
       </c>
     </row>
     <row r="3">
@@ -881,7 +852,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -895,21 +866,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Dependency installation failed</t>
+          <t>General Stress Test (unrecognized dependencies)</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -923,21 +894,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>edge_case_input</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Env Validation (dotenv)</t>
+          <t>General Stress Test (unrecognized dependencies)</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -954,18 +925,14 @@
           <t>warning</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>data_volume_scaling</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Computation Coupling (App wait for timeout)</t>
+          <t>1 missing dependency</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -979,21 +946,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>memory_profiling</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cache Memory Growth (streamlit)</t>
+          <t>Data Volume Scaling (pandas)</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8">
@@ -1007,21 +974,21 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>memory_profiling</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Data Volume Scaling (pandas)</t>
+          <t>Cache Memory Growth (streamlit)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>50</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
@@ -1035,21 +1002,21 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>memory_profiling</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Array Size Scaling (numpy)</t>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>19</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10">
@@ -1063,7 +1030,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1073,11 +1040,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Data Volume Scaling (pandas)</t>
+          <t>Array Size Scaling (numpy)</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
@@ -1101,13 +1068,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1115,27 +1082,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>memory_profiling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
+          <t>Application server could not start</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>96</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1148,22 +1115,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Scenario failed: pandas_iterrows_vs_vectorized</t>
+          <t>Dependency installation failed</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1171,27 +1138,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Scenario failed: numpy_matrix_operation_scaling</t>
+          <t>Response time degradation on your application</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1199,27 +1166,23 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>data_volume_scaling</t>
-        </is>
-      </c>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Scenario failed: pandas_merge_memory_stress</t>
+          <t>1 missing dependency</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1227,21 +1190,21 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>edge_case_input</t>
+          <t>concurrent_execution</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Scenario failed: pandas_edge_case_dtypes</t>
+          <t>Ssr Concurrent Load (nextjs)</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1269,7 +1232,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18">
@@ -1293,11 +1256,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Array Size Scaling (numpy)</t>
+          <t>Data Volume Scaling (pandas)</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -1321,11 +1284,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Data Volume Scaling (pandas)</t>
+          <t>Array Size Scaling (numpy)</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -1342,14 +1305,18 @@
           <t>warning</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1 missing dependency</t>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -1373,13 +1340,13 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1387,27 +1354,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>memory_profiling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Cache Memory Growth (streamlit)</t>
+          <t>Application server could not start</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1415,27 +1382,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>memory_profiling</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Application server could not start</t>
+          <t>Cache Memory Growth (streamlit)</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1453,13 +1420,13 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1467,27 +1434,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Data Volume Scaling (pandas)</t>
+          <t>Response time degradation on your application</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1501,17 +1468,17 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4 missing dependencies</t>
+          <t>2 missing dependencies</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1519,27 +1486,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>memory_profiling</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Application server could not start</t>
+          <t>Cache Memory Growth (streamlit)</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1552,22 +1519,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>memory_profiling</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Response time degradation on your application</t>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1575,27 +1542,23 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>http_load_testing</t>
-        </is>
-      </c>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Dependency installation failed</t>
+          <t>2 missing dependencies</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1603,27 +1566,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>data_volume_scaling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Computation Coupling (Abort signal timeout)</t>
+          <t>Application server could not start</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1634,24 +1597,20 @@
           <t>warning</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>concurrent_execution</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>API Coupling (Src components projects submission wizard submit project)</t>
+          <t>3 missing dependencies</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1659,27 +1618,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>memory_profiling</t>
+          <t>http_load_testing</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Cache Memory Growth (streamlit)</t>
+          <t>Application server could not start</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1687,27 +1646,23 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>http_load_testing</t>
-        </is>
-      </c>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Application server could not start</t>
+          <t>1 missing dependency</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1720,22 +1675,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Dependency installation failed</t>
+          <t>N Plus One Detection (sqlalchemy)</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1748,22 +1703,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>concurrent_execution</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Rate Limit Stress (openai)</t>
+          <t>N Plus One Detection (sqlalchemy)</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1771,7 +1726,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1781,17 +1736,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Computation Coupling (Clear timeout)</t>
+          <t>Validation Throughput (pydantic)</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1813,13 +1768,13 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1837,17 +1792,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>N Plus One Detection (sqlalchemy)</t>
+          <t>General Stress Test (unrecognized dependencies)</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1855,7 +1810,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1865,17 +1820,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>API Coupling (App analyzers package fetcher  fetch from github)</t>
+          <t>Concurrent Request Load (requests)</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1883,27 +1838,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>http_load_testing</t>
+          <t>data_volume_scaling</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Application degrades under concurrent load</t>
+          <t>Computation Coupling (Clear timeout)</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1911,7 +1866,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1921,151 +1876,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Get Root (http)</t>
+          <t>Dependency installation failed</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>http_load_testing</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Application server could not start</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
         <v>2</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>data_volume_scaling</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>General Stress Test (unrecognized dependencies)</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>concurrent_execution</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>API Coupling (Src cursorx download and extract)</t>
-        </is>
-      </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>edge_case_input</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Env Validation (dotenv)</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>5</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>concurrent_execution</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Concurrent Request Load (requests)</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2079,12 +1894,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -2125,7 +1940,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>509</v>
+        <v>924</v>
       </c>
     </row>
     <row r="3">
@@ -2143,7 +1958,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -2157,11 +1972,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>express</t>
+          <t>flask</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -2175,11 +1990,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>dotenv</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -2193,11 +2008,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>http</t>
+          <t>express</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -2211,11 +2026,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>streamlit</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>180</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8">
@@ -2229,11 +2044,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>streamlit</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>86</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9">
@@ -2251,7 +2066,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>36</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10">
@@ -2269,7 +2084,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>18</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11">
@@ -2283,17 +2098,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pyarrow</t>
+          <t>uvicorn</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2301,17 +2116,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>npm-start</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>370</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2319,17 +2134,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>nextjs</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>174</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2337,17 +2152,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>requests</t>
+          <t>express</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>119</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2355,17 +2170,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>streamlit</t>
+          <t>fletzxing</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>portfolio</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2373,11 +2188,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>plotly</t>
+          <t>react</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2391,11 +2206,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>streamlit</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>32</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18">
@@ -2409,11 +2224,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19">
@@ -2427,11 +2242,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>streamlit</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>14</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20">
@@ -2449,7 +2264,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21">
@@ -2463,17 +2278,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>seaborn</t>
+          <t>scipy</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2481,17 +2296,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>streamlit</t>
+          <t>fastapi</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2499,17 +2314,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>pandas</t>
+          <t>uvicorn</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2517,17 +2332,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>streamlit</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2535,17 +2350,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tensorflow</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2553,17 +2368,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>scikit-learn</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2571,17 +2386,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>npm-start</t>
+          <t>pandas</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2589,17 +2404,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>nextjs</t>
+          <t>streamlit</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2607,17 +2422,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>react</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2625,17 +2440,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>react-dom</t>
+          <t>scikit-learn</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>portfolio</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2643,17 +2458,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>tailwindcss</t>
+          <t>joblib</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2661,17 +2476,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>streamlit</t>
+          <t>fastapi</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2679,17 +2494,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>express</t>
+          <t>uvicorn</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2697,17 +2512,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>fastapi</t>
+          <t>sqlalchemy</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2715,17 +2530,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>uvicorn</t>
+          <t>http</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>chatbot</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2733,17 +2548,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>psycopg2-binary</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2751,17 +2566,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>fastapi</t>
+          <t>npm-start</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2769,17 +2584,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>uvicorn</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2787,7 +2602,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>http</t>
+          <t>dotenv</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2797,7 +2612,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2805,17 +2620,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>npm-start</t>
+          <t>express</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2823,64 +2638,10 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sqlalchemy</t>
+          <t>tomli</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>npm-start</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>dotenv</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>requests</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2895,7 +2656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2921,7 +2682,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>575</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="3">
@@ -2931,57 +2692,57 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>178</v>
+        <v>503</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>api_service</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>api_service</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>data_pipeline</t>
+          <t>ml_model</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ml_model</t>
+          <t>data_pipeline</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>utility</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2991,16 +2752,6 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>chatbot</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3015,7 +2766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3025,9 +2776,8 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3068,15 +2818,10 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>utility</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>web_app</t>
         </is>
@@ -3089,13 +2834,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3</v>
+        <v>39</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -3105,25 +2850,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>22</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -3133,19 +2878,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>143</v>
+        <v>364</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -3155,99 +2906,1935 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>71</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>31</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>13</v>
+      </c>
+      <c r="I5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ml_model</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>46</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>27</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>portfolio</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>37</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>web_app</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1062</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Business Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>With Issues</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Clean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Failure Rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Deps Seen</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Deps Failed</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Dep Fail Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1582</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1482</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>93.7%</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1791</v>
+      </c>
+      <c r="G2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>265</v>
+      </c>
+      <c r="C3" t="n">
+        <v>244</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>92.1%</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>746</v>
+      </c>
+      <c r="G3" t="n">
+        <v>140</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>18.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>112</v>
+      </c>
+      <c r="C4" t="n">
+        <v>95</v>
+      </c>
+      <c r="D4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>84.8%</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>577</v>
+      </c>
+      <c r="G4" t="n">
+        <v>86</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>14.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>67</v>
+      </c>
+      <c r="C5" t="n">
+        <v>57</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>85.1%</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>784</v>
+      </c>
+      <c r="G5" t="n">
+        <v>76</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>36</v>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>83.3%</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>308</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>88.9%</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>184</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>80.0%</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>105</v>
+      </c>
+      <c r="G8" t="n">
+        <v>14</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>76</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>climate</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>75</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2.7%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Business Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Data Volume Scaling (pandas)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Response time degradation on your application</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1 missing dependency</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Data Volume Scaling (pandas)</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1 missing dependency</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Response time degradation on your application</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Data Volume Scaling (pandas)</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1 missing dependency</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2 missing dependencies</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>General Stress Test (unrecognized dependencies)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Failure indicators triggered: streamlit_cache_memory_growth</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Data Volume Scaling (pandas)</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Response time degradation on your application</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Array Size Scaling (numpy)</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3 missing dependencies</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1 missing dependency</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>3 missing dependencies</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2 missing dependencies</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>General Stress Test (unrecognized dependencies)</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Array Size Scaling (numpy)</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Response time degradation on your application</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>7 missing dependencies</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>concurrent_execution</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Concurrent Request Load (requests)</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Array Size Scaling (numpy)</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Endpoint /narratives/1 degrades under concurrent load</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Get Narratives 1 (http)</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Get Trends 1 (http)</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>climate</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>data_volume_scaling</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Array Size Scaling (numpy)</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>climate</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>http_load_testing</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Application server could not start</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>climate</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>memory_profiling</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Cache Memory Growth (streamlit)</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Business Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>api_service</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>chatbot</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ml_model</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>portfolio</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>utility</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>web_app</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ai_assistant</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>53</v>
+      </c>
+      <c r="D2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>climate</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>data_science</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D4" t="n">
+        <v>127</v>
+      </c>
+      <c r="E4" t="n">
+        <v>41</v>
+      </c>
+      <c r="F4" t="n">
+        <v>76</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>developer_tools</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
       </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
       <c r="I5" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ml_model</t>
-        </is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>portfolio</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>23</v>
+          <t>fintech</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>unclassified</t>
-        </is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>35</v>
+      </c>
+      <c r="C8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" t="n">
+        <v>246</v>
+      </c>
+      <c r="E8" t="n">
+        <v>58</v>
+      </c>
+      <c r="F8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>142</v>
       </c>
       <c r="H8" t="n">
-        <v>110</v>
+        <v>34</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1045</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>utility</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>7</v>
-      </c>
-      <c r="J9" t="n">
+          <t>healthcare</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>web_app</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+          <t>social_media</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
         <v>2</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>